<commit_message>
nova estrutura da tabela produtos adaptada nas views produtos e show
</commit_message>
<xml_diff>
--- a/Quadro.kanban.metricas.xlsx
+++ b/Quadro.kanban.metricas.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carolina\Desktop\CROFLINE\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\Crofline\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9264" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9270"/>
   </bookViews>
   <sheets>
     <sheet name="QUADO-KANBAN" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>A FAZER</t>
   </si>
@@ -111,6 +111,9 @@
   </si>
   <si>
     <t>Ideia da IA</t>
+  </si>
+  <si>
+    <t>preencher</t>
   </si>
 </sst>
 </file>
@@ -324,6 +327,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="16" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -340,9 +346,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -372,22 +375,22 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1191869</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>49182</xdr:rowOff>
+      <xdr:colOff>1084712</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>13464</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>2982569</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>79662</xdr:rowOff>
+      <xdr:colOff>2875412</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>43943</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="2" name="CaixaDeTexto 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{74E5234A-B335-4EE2-9915-DE5519AAEA2C}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{74E5234A-B335-4EE2-9915-DE5519AAEA2C}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -395,8 +398,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5306669" y="839757"/>
-          <a:ext cx="1790700" cy="1230630"/>
+          <a:off x="5204275" y="2787620"/>
+          <a:ext cx="1790700" cy="1280636"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -529,7 +532,7 @@
         <xdr:cNvPr id="3" name="CaixaDeTexto 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{53239B3F-6370-4DC2-9876-EE3113BDE0C3}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{53239B3F-6370-4DC2-9876-EE3113BDE0C3}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -690,7 +693,7 @@
         <xdr:cNvPr id="4" name="CaixaDeTexto 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{A27257E5-52BD-4C91-9F79-B670FFD59A29}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A27257E5-52BD-4C91-9F79-B670FFD59A29}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -816,23 +819,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>2190874</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>93320</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>964530</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>57601</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>3981574</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>112370</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2755230</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>76651</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="5" name="CaixaDeTexto 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{20B8EB74-ED9D-4484-A492-C51932F4FEB5}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{20B8EB74-ED9D-4484-A492-C51932F4FEB5}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -840,8 +843,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2190874" y="2255495"/>
-          <a:ext cx="1790700" cy="1219200"/>
+          <a:off x="5084093" y="1045820"/>
+          <a:ext cx="1790700" cy="1269206"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -901,7 +904,7 @@
               <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t> Planejar json de cores e tamanhos dos produtos</a:t>
+            <a:t> Mudar campo qtd_detalhes para detalhes, e add chaves imagens, valor e qtd</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="pt-BR" sz="1100" b="1">
@@ -974,7 +977,7 @@
         <xdr:cNvPr id="6" name="CaixaDeTexto 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{B3B6A202-3707-41BE-BFF0-E830FFF85602}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B3B6A202-3707-41BE-BFF0-E830FFF85602}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1154,7 +1157,7 @@
         <xdr:cNvPr id="8" name="CaixaDeTexto 7">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{A27257E5-52BD-4C91-9F79-B670FFD59A29}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A27257E5-52BD-4C91-9F79-B670FFD59A29}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1296,7 +1299,7 @@
         <xdr:cNvPr id="9" name="CaixaDeTexto 8">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{A27257E5-52BD-4C91-9F79-B670FFD59A29}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A27257E5-52BD-4C91-9F79-B670FFD59A29}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1441,23 +1444,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>133350</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1097756</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>164308</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1924050</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>2888456</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>4764</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="10" name="CaixaDeTexto 9">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{A27257E5-52BD-4C91-9F79-B670FFD59A29}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A27257E5-52BD-4C91-9F79-B670FFD59A29}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1465,8 +1468,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="133350" y="3886200"/>
-          <a:ext cx="1790700" cy="1219200"/>
+          <a:off x="13456444" y="2402683"/>
+          <a:ext cx="1790700" cy="1269206"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1618,7 +1621,7 @@
         <xdr:cNvPr id="11" name="CaixaDeTexto 10">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{A27257E5-52BD-4C91-9F79-B670FFD59A29}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A27257E5-52BD-4C91-9F79-B670FFD59A29}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1760,7 +1763,7 @@
         <xdr:cNvPr id="12" name="CaixaDeTexto 11">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{A27257E5-52BD-4C91-9F79-B670FFD59A29}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A27257E5-52BD-4C91-9F79-B670FFD59A29}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1921,7 +1924,7 @@
         <xdr:cNvPr id="13" name="CaixaDeTexto 12">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{A27257E5-52BD-4C91-9F79-B670FFD59A29}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A27257E5-52BD-4C91-9F79-B670FFD59A29}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2082,7 +2085,7 @@
         <xdr:cNvPr id="14" name="CaixaDeTexto 13">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{A27257E5-52BD-4C91-9F79-B670FFD59A29}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A27257E5-52BD-4C91-9F79-B670FFD59A29}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2223,7 +2226,7 @@
         <xdr:cNvPr id="15" name="CaixaDeTexto 14">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{A27257E5-52BD-4C91-9F79-B670FFD59A29}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A27257E5-52BD-4C91-9F79-B670FFD59A29}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2690,7 +2693,7 @@
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="54" style="1" customWidth="1"/>
     <col min="2" max="2" width="54" style="2" customWidth="1"/>
@@ -2698,23 +2701,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18.75">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="15"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="16"/>
     </row>
     <row r="2" spans="1:4" ht="12" customHeight="1">
-      <c r="A2" s="16" t="str">
+      <c r="A2" s="17" t="str">
         <f ca="1">"Atualizado em: " &amp; TEXT(NOW(),"dd/mm/aaaa hh:mm")</f>
-        <v>Atualizado em: 17/03/2026 20:44</v>
-      </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="18"/>
-    </row>
-    <row r="3" spans="1:4" ht="18">
+        <v>Atualizado em: 11/04/2026 23:09</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="19"/>
+    </row>
+    <row r="3" spans="1:4" ht="18.75">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
@@ -2745,12 +2748,12 @@
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
   <dimension ref="A1:H45"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="8" width="23.296875" style="8" customWidth="1"/>
+    <col min="1" max="8" width="23.25" style="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18">
+    <row r="1" spans="1:8" ht="18.75">
       <c r="A1" s="6" t="s">
         <v>5</v>
       </c>
@@ -2855,7 +2858,7 @@
       <c r="B5" s="10">
         <v>46098</v>
       </c>
-      <c r="C5" s="19">
+      <c r="C5" s="13">
         <v>46137</v>
       </c>
       <c r="D5" s="9"/>
@@ -2868,10 +2871,10 @@
       <c r="A6" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="19">
+      <c r="B6" s="13">
         <v>46098</v>
       </c>
-      <c r="C6" s="19">
+      <c r="C6" s="13">
         <v>46132</v>
       </c>
       <c r="D6" s="9"/>
@@ -2884,10 +2887,10 @@
       <c r="A7" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="19">
+      <c r="B7" s="13">
         <v>46098</v>
       </c>
-      <c r="C7" s="19">
+      <c r="C7" s="13">
         <v>46122</v>
       </c>
       <c r="D7" s="9"/>
@@ -2900,14 +2903,16 @@
       <c r="A8" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="19">
+      <c r="B8" s="13">
         <v>46098</v>
       </c>
-      <c r="C8" s="19">
+      <c r="C8" s="13">
         <v>46109</v>
       </c>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
+      <c r="D8" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" s="13"/>
       <c r="F8" s="9"/>
       <c r="G8" s="9"/>
       <c r="H8" s="9"/>
@@ -2916,10 +2921,10 @@
       <c r="A9" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="19">
+      <c r="B9" s="13">
         <v>46098</v>
       </c>
-      <c r="C9" s="19">
+      <c r="C9" s="13">
         <v>46142</v>
       </c>
       <c r="D9" s="9"/>
@@ -2932,10 +2937,10 @@
       <c r="A10" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="19">
+      <c r="B10" s="13">
         <v>46098</v>
       </c>
-      <c r="C10" s="19">
+      <c r="C10" s="13">
         <v>46147</v>
       </c>
       <c r="D10" s="9"/>
@@ -2948,10 +2953,10 @@
       <c r="A11" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="19">
+      <c r="B11" s="13">
         <v>46098</v>
       </c>
-      <c r="C11" s="19">
+      <c r="C11" s="13">
         <v>46147</v>
       </c>
       <c r="D11" s="9"/>
@@ -2964,10 +2969,10 @@
       <c r="A12" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B12" s="19">
+      <c r="B12" s="13">
         <v>46098</v>
       </c>
-      <c r="C12" s="19">
+      <c r="C12" s="13">
         <v>46142</v>
       </c>
       <c r="D12" s="9"/>
@@ -2980,10 +2985,10 @@
       <c r="A13" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="19">
+      <c r="B13" s="13">
         <v>46098</v>
       </c>
-      <c r="C13" s="19">
+      <c r="C13" s="13">
         <v>46162</v>
       </c>
       <c r="D13" s="9"/>
@@ -3082,7 +3087,7 @@
       <c r="G22" s="11"/>
       <c r="H22" s="11"/>
     </row>
-    <row r="23" spans="1:8" ht="15">
+    <row r="23" spans="1:8">
       <c r="A23" s="7"/>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
@@ -3092,7 +3097,7 @@
       <c r="G23" s="7"/>
       <c r="H23" s="7"/>
     </row>
-    <row r="24" spans="1:8" ht="15">
+    <row r="24" spans="1:8">
       <c r="A24" s="7"/>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
@@ -3102,7 +3107,7 @@
       <c r="G24" s="7"/>
       <c r="H24" s="7"/>
     </row>
-    <row r="25" spans="1:8" ht="15">
+    <row r="25" spans="1:8">
       <c r="A25" s="7"/>
       <c r="B25" s="7"/>
       <c r="C25" s="7"/>
@@ -3112,7 +3117,7 @@
       <c r="G25" s="7"/>
       <c r="H25" s="7"/>
     </row>
-    <row r="26" spans="1:8" ht="15">
+    <row r="26" spans="1:8">
       <c r="A26" s="7"/>
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
@@ -3122,7 +3127,7 @@
       <c r="G26" s="7"/>
       <c r="H26" s="7"/>
     </row>
-    <row r="27" spans="1:8" ht="15">
+    <row r="27" spans="1:8">
       <c r="A27" s="7"/>
       <c r="B27" s="7"/>
       <c r="C27" s="7"/>
@@ -3132,7 +3137,7 @@
       <c r="G27" s="7"/>
       <c r="H27" s="7"/>
     </row>
-    <row r="28" spans="1:8" ht="15">
+    <row r="28" spans="1:8">
       <c r="A28" s="7"/>
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>

</xml_diff>